<commit_message>
added data to all choctaw list
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By Blood.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Cherokee/Cherokee By Blood.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ID</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>Source</t>
+  </si>
+  <si>
+    <t>Link</t>
   </si>
 </sst>
 </file>
@@ -387,10 +390,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -432,6 +435,9 @@
       </c>
       <c r="N1" t="s">
         <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>